<commit_message>
feat: finish player_data implementation
</commit_message>
<xml_diff>
--- a/Main/Statistics/PlayerData.xlsx
+++ b/Main/Statistics/PlayerData.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -464,11 +464,6 @@
           <t>total_seconds_played</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>completed_data</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -488,7 +483,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>"uBt</t>
+          <t>"u"t</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -498,17 +493,12 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>:D</t>
+          <t xml:space="preserve"> u</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>RhoBH:V"RxObrOKauh</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>lisXw8S8TVnhsbKaVebxTV"BtaR8qwhKkMsCVo6HaDJOK V2sHaKTfzDsrqr,hJcwOTXB8CbsTFgDBO.,isX78S8lVnD"bH V"s7:DhT7Y4kTyai{fKg 26V:hslKDVrgH"oTfzDshqr,D2cHOKslxCcQ68TbTfzDs"qr,b2c7:brT8CT2Ox"b2Zs8hUbzG4"R/OcesK:DQTt"b"t.,isXa8S8O7ncBRKTXhTHaDsbaY4k6yDi{fwguolwRcJRx"hXsKCR8qVhbkMsRVoTx he68aDQ6x:TTfzCsXqr,c2cwRVB6wOcebHgcJR.,iQX88S8OxnTrTwgoeO7ChJgFY4k6y:i{fVa eltCurTtRusgw:cTfzCs2qr,hss/gV2gKDbs68:heO.,iQXa8S86tnue68guQg8:bJsKTR8qKhKkMsOco6VgoXRFacBga"ohZs8bUlzG4QB/DoJg7TuJT8gDJtxY4klyRi{fVg "tagussw:DsRxCR8qKhckMsCKosVRbh6tToQOa chZs8bURzG4hB/OKB6wCT"bHOo"Zs8bUBzG4XO/TXBgtOhQstRu2g7Y4klyDi{fVODolF:h2B8:KJOVaR8qVhKkMsDh2cKgD2BF:hrsH DrZs8KUBzG4Js/aVXOwCXelHRVJZs8TUTzG4rt/RKeT7guQBa"V2b.,iXX78S8RxnXrOwDo2baRuXl{</t>
+          <t>O Q6FabrTtCurt8CKB</t>
         </is>
       </c>
     </row>
@@ -548,9 +538,115 @@
           <t>CrcHHpXlH/42b8O"B</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>6kTyiU{f7l1hTFiN2bFiqhOKF{8qVNqkMsHpobalNJs7O4hbw9qrZsJ.UTzhhrl//CeOK/qBbxKNQt{</t>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Hello</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>6Y  L</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>ka</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>ki7</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>k</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>ka</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>1Qi1ai0l1ww7k0w0k</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>p</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>d</t>
         </is>
       </c>
     </row>

</xml_diff>